<commit_message>
Updated billing and dashboard changes
</commit_message>
<xml_diff>
--- a/tokens.xlsx
+++ b/tokens.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,7 +449,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>P Rizwana</t>
+          <t>RIZWANA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,12 +474,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P Rizwana</t>
+          <t>abbas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>7382132251</t>
+          <t>9988776655</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -499,22 +499,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P Rizwana</t>
+          <t>shiva</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7382132251</t>
+          <t>9876543245</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>manish</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>8978685466</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Waiting</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>App</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Walk-in</t>
         </is>
       </c>
     </row>

</xml_diff>